<commit_message>
Web Push bildirimleri: sabah/akşam otomasyon + hedef barlar
- sw.js: push event listener + notificationclick handler eklendi
- bist_tracker.html: VAPID key, initPush(), sendPushNotify() eklendi
  Hedef bar ve TAKİP bar %100'e ulaşınca Firebase pushQueue'ya yazar
- automation_server.pyw: send_push_to_all(), _check_push_queue(),
  /api/notify endpoint eklendi. pushQueue her 10s kontrol ediliyor.
- morning_automation.pyw: tamamlanınca /api/notify çağırır
- evening_automation.pyw: tamamlanınca /api/notify çağırır

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ATR_Sonuc.xlsx
+++ b/ATR_Sonuc.xlsx
@@ -549,25 +549,25 @@
         <x:v>17.45</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>0.0536</x:v>
+        <x:v>0.0321</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>0.1821</x:v>
+        <x:v>0.1864</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>0.2386</x:v>
+        <x:v>0.23</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>0.295</x:v>
+        <x:v>0.2957</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.68</x:v>
+        <x:v>0.6643</x:v>
       </x:c>
       <x:c r="J2" s="0">
         <x:v>1.8114</x:v>
       </x:c>
       <x:c r="K2" s="0">
-        <x:v>0.5435</x:v>
+        <x:v>0.5367</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:11">
@@ -581,28 +581,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>75.75</x:v>
+        <x:v>75.1</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>0.0821</x:v>
+        <x:v>0.175</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>0.7893</x:v>
+        <x:v>0.8607</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>1.0179</x:v>
+        <x:v>1.0786</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>1.2964</x:v>
+        <x:v>1.325</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>2.9642</x:v>
+        <x:v>2.9195</x:v>
       </x:c>
       <x:c r="J3" s="0">
         <x:v>7.6001</x:v>
       </x:c>
       <x:c r="K3" s="0">
-        <x:v>2.2917</x:v>
+        <x:v>2.3265</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:11">
@@ -616,28 +616,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>362.25</x:v>
+        <x:v>375.25</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>1.1071</x:v>
+        <x:v>1.1607</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>4.75</x:v>
+        <x:v>6.1071</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>5.6429</x:v>
+        <x:v>6.3393</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>6.4286</x:v>
+        <x:v>6.8929</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>13.5</x:v>
+        <x:v>13.7857</x:v>
       </x:c>
       <x:c r="J4" s="0">
-        <x:v>31.4857</x:v>
+        <x:v>32.3786</x:v>
       </x:c>
       <x:c r="K4" s="0">
-        <x:v>10.4857</x:v>
+        <x:v>11.1107</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:11">
@@ -651,28 +651,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>207.3</x:v>
+        <x:v>209.1</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>0.5143</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>2.6643</x:v>
+        <x:v>3.1143</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>2.9929</x:v>
+        <x:v>3.45</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>3.5643</x:v>
+        <x:v>3.8786</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>10.2929</x:v>
+        <x:v>10.3857</x:v>
       </x:c>
       <x:c r="J5" s="0">
         <x:v>21.4071</x:v>
       </x:c>
       <x:c r="K5" s="0">
-        <x:v>6.906</x:v>
+        <x:v>7.1143</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:11">
@@ -686,28 +686,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>726.5</x:v>
+        <x:v>739</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>2.0714</x:v>
+        <x:v>1.5714</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>7.25</x:v>
+        <x:v>8.3214</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>8.25</x:v>
+        <x:v>9.4643</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>10.1786</x:v>
+        <x:v>10.7143</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>24.7143</x:v>
+        <x:v>23.8929</x:v>
       </x:c>
       <x:c r="J6" s="0">
-        <x:v>56.8571</x:v>
+        <x:v>57</x:v>
       </x:c>
       <x:c r="K6" s="0">
-        <x:v>18.2202</x:v>
+        <x:v>18.494</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -721,28 +721,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>2002</x:v>
+        <x:v>1999</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>5.2143</x:v>
+        <x:v>2.7857</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>17.2857</x:v>
+        <x:v>21.7143</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>19.1429</x:v>
+        <x:v>20.2857</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>21.1429</x:v>
+        <x:v>22.3571</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>54.7143</x:v>
+        <x:v>49.7143</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>175.4286</x:v>
       </x:c>
       <x:c r="K7" s="0">
-        <x:v>48.8214</x:v>
+        <x:v>48.7143</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:11">
@@ -756,28 +756,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>20.62</x:v>
+        <x:v>20.5</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>0.0829</x:v>
+        <x:v>0.0443</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>0.2507</x:v>
+        <x:v>0.265</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>0.2786</x:v>
+        <x:v>0.2893</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>0.3386</x:v>
+        <x:v>0.3421</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.7657</x:v>
+        <x:v>0.7686</x:v>
       </x:c>
       <x:c r="J8" s="0">
         <x:v>2.0614</x:v>
       </x:c>
       <x:c r="K8" s="0">
-        <x:v>0.6296</x:v>
+        <x:v>0.6285</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
@@ -791,28 +791,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>95.05</x:v>
+        <x:v>94.75</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>0.2179</x:v>
+        <x:v>0.1464</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>0.9592</x:v>
+        <x:v>1.0429</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>1.1512</x:v>
+        <x:v>1.1773</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.2883</x:v>
+        <x:v>1.3268</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>3.0212</x:v>
+        <x:v>2.8979</x:v>
       </x:c>
       <x:c r="J9" s="0">
         <x:v>6.81</x:v>
       </x:c>
       <x:c r="K9" s="0">
-        <x:v>2.2413</x:v>
+        <x:v>2.2335</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:11">
@@ -826,28 +826,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>29.58</x:v>
+        <x:v>30.46</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>0.0629</x:v>
+        <x:v>0.1086</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>0.2843</x:v>
+        <x:v>0.3414</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>0.3829</x:v>
+        <x:v>0.4243</x:v>
       </x:c>
       <x:c r="H10" s="0">
-        <x:v>0.5314</x:v>
+        <x:v>0.5943</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>1.0971</x:v>
+        <x:v>1.1357</x:v>
       </x:c>
       <x:c r="J10" s="0">
-        <x:v>2.0657</x:v>
+        <x:v>2.0771</x:v>
       </x:c>
       <x:c r="K10" s="0">
-        <x:v>0.7374</x:v>
+        <x:v>0.7802</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:11">
@@ -861,28 +861,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>101.8</x:v>
+        <x:v>102.2</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>0.3</x:v>
+        <x:v>0.2357</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>0.9214</x:v>
+        <x:v>1.1357</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>1.0464</x:v>
+        <x:v>1.1607</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1.225</x:v>
+        <x:v>1.3464</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>3.6643</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="J11" s="0">
         <x:v>8.648</x:v>
       </x:c>
       <x:c r="K11" s="0">
-        <x:v>2.6342</x:v>
+        <x:v>2.6544</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:11">
@@ -896,28 +896,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>137.5</x:v>
+        <x:v>136.5</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>0.4286</x:v>
+        <x:v>0.2571</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1.85</x:v>
+        <x:v>1.8929</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>2.0952</x:v>
+        <x:v>2.1558</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>2.5127</x:v>
+        <x:v>2.5225</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>4.6398</x:v>
+        <x:v>4.6531</x:v>
       </x:c>
       <x:c r="J12" s="0">
         <x:v>11.467</x:v>
       </x:c>
       <x:c r="K12" s="0">
-        <x:v>3.8322</x:v>
+        <x:v>3.8247</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:11">
@@ -931,28 +931,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>483.25</x:v>
+        <x:v>494.5</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>1.3571</x:v>
+        <x:v>1.1964</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>6.3571</x:v>
+        <x:v>7.5536</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>7.25</x:v>
+        <x:v>7.9821</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>9.5893</x:v>
+        <x:v>10.5893</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>21.8214</x:v>
+        <x:v>21.6786</x:v>
       </x:c>
       <x:c r="J13" s="0">
         <x:v>52.75</x:v>
       </x:c>
       <x:c r="K13" s="0">
-        <x:v>16.5208</x:v>
+        <x:v>16.9583</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:11">
@@ -966,28 +966,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>14.09</x:v>
+        <x:v>14.15</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>0.0471</x:v>
+        <x:v>0.0357</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>0.1929</x:v>
+        <x:v>0.2121</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>0.2093</x:v>
+        <x:v>0.2214</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>0.23</x:v>
+        <x:v>0.2371</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.4924</x:v>
+        <x:v>0.4917</x:v>
       </x:c>
       <x:c r="J14" s="0">
         <x:v>1.2753</x:v>
       </x:c>
       <x:c r="K14" s="0">
-        <x:v>0.4078</x:v>
+        <x:v>0.4122</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:11">
@@ -1001,28 +1001,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>201.4</x:v>
+        <x:v>200.3</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>0.5714</x:v>
+        <x:v>0.3214</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>2.2357</x:v>
+        <x:v>2.3786</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>2.5357</x:v>
+        <x:v>2.6571</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>2.5643</x:v>
+        <x:v>2.7643</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>6.2728</x:v>
+        <x:v>6.0816</x:v>
       </x:c>
       <x:c r="J15" s="0">
         <x:v>13.9501</x:v>
       </x:c>
       <x:c r="K15" s="0">
-        <x:v>4.6883</x:v>
+        <x:v>4.6922</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:11">
@@ -1036,28 +1036,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>34.38</x:v>
+        <x:v>36.84</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>0.1057</x:v>
+        <x:v>0.1729</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>0.4343</x:v>
+        <x:v>0.7114</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>0.5914</x:v>
+        <x:v>0.7329</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>0.7257</x:v>
+        <x:v>0.93</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>1.3829</x:v>
+        <x:v>1.5771</x:v>
       </x:c>
       <x:c r="J16" s="0">
-        <x:v>2.6</x:v>
+        <x:v>2.7871</x:v>
       </x:c>
       <x:c r="K16" s="0">
-        <x:v>0.9733</x:v>
+        <x:v>1.1519</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:11">
@@ -1071,28 +1071,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>627.5</x:v>
+        <x:v>646</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>1.9286</x:v>
+        <x:v>1.3214</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>6.4643</x:v>
+        <x:v>7.8571</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>6.8929</x:v>
+        <x:v>8.3214</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>8</x:v>
+        <x:v>9.4286</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>19.1071</x:v>
+        <x:v>19.9643</x:v>
       </x:c>
       <x:c r="J17" s="0">
-        <x:v>50.5714</x:v>
+        <x:v>51.1429</x:v>
       </x:c>
       <x:c r="K17" s="0">
-        <x:v>15.494</x:v>
+        <x:v>16.3393</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:11">
@@ -1106,28 +1106,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>42.76</x:v>
+        <x:v>42.14</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>0.24</x:v>
+        <x:v>0.0829</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>0.75</x:v>
+        <x:v>0.6071</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>0.7771</x:v>
+        <x:v>0.7514</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>0.9471</x:v>
+        <x:v>0.9129</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>2.3043</x:v>
+        <x:v>2.1971</x:v>
       </x:c>
       <x:c r="J18" s="0">
         <x:v>4.3829</x:v>
       </x:c>
       <x:c r="K18" s="0">
-        <x:v>1.5669</x:v>
+        <x:v>1.489</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:11">
@@ -1141,28 +1141,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>20.8</x:v>
+        <x:v>20.94</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>0.1443</x:v>
+        <x:v>0.0629</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>0.3543</x:v>
+        <x:v>0.3557</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>0.4921</x:v>
+        <x:v>0.4529</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>0.5421</x:v>
+        <x:v>0.5179</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>1.2686</x:v>
+        <x:v>1.2571</x:v>
       </x:c>
       <x:c r="J19" s="0">
         <x:v>1.8579</x:v>
       </x:c>
       <x:c r="K19" s="0">
-        <x:v>0.7765</x:v>
+        <x:v>0.7507</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:11">
@@ -1176,28 +1176,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>186</x:v>
+        <x:v>184.5</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>0.5286</x:v>
+        <x:v>0.2643</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>2.2786</x:v>
+        <x:v>2.3143</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>2.4357</x:v>
+        <x:v>2.45</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>2.6143</x:v>
+        <x:v>2.6786</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>5.2143</x:v>
+        <x:v>5.25</x:v>
       </x:c>
       <x:c r="J20" s="0">
         <x:v>13.6286</x:v>
       </x:c>
       <x:c r="K20" s="0">
-        <x:v>4.45</x:v>
+        <x:v>4.431</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:11">
@@ -1211,28 +1211,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>96.35</x:v>
+        <x:v>97.3</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>0.2857</x:v>
+        <x:v>0.2429</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1.2429</x:v>
+        <x:v>1.4036</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>1.5214</x:v>
+        <x:v>1.5464</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1.6643</x:v>
+        <x:v>1.7786</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>3.3783</x:v>
+        <x:v>3.4332</x:v>
       </x:c>
       <x:c r="J21" s="0">
         <x:v>8.2544</x:v>
       </x:c>
       <x:c r="K21" s="0">
-        <x:v>2.7245</x:v>
+        <x:v>2.7765</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:11">
@@ -1246,28 +1246,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>2.48</x:v>
+        <x:v>2.46</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>0.0121</x:v>
+        <x:v>0.0136</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>0.0336</x:v>
+        <x:v>0.0329</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>0.0414</x:v>
+        <x:v>0.0357</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>0.0521</x:v>
+        <x:v>0.0514</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.0986</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="J22" s="0">
         <x:v>0.2714</x:v>
       </x:c>
       <x:c r="K22" s="0">
-        <x:v>0.0849</x:v>
+        <x:v>0.0842</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:11">
@@ -1281,28 +1281,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>46.7</x:v>
+        <x:v>46.4</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>0.1571</x:v>
+        <x:v>0.1086</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>0.6743</x:v>
+        <x:v>0.6814</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>0.7414</x:v>
+        <x:v>0.76</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>0.7857</x:v>
+        <x:v>0.7986</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>2.31</x:v>
+        <x:v>2.1186</x:v>
       </x:c>
       <x:c r="J23" s="0">
         <x:v>4.2871</x:v>
       </x:c>
       <x:c r="K23" s="0">
-        <x:v>1.4926</x:v>
+        <x:v>1.459</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:11">
@@ -1316,28 +1316,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>344</x:v>
+        <x:v>337.75</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>0.5536</x:v>
+        <x:v>0.6429</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>4.625</x:v>
+        <x:v>5.3393</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>5.6071</x:v>
+        <x:v>5.9643</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>7.0357</x:v>
+        <x:v>7.1071</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>14.4107</x:v>
+        <x:v>14.7143</x:v>
       </x:c>
       <x:c r="J24" s="0">
         <x:v>27.7143</x:v>
       </x:c>
       <x:c r="K24" s="0">
-        <x:v>9.9911</x:v>
+        <x:v>10.247</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:11">
@@ -1351,28 +1351,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>111.2</x:v>
+        <x:v>112.3</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>0.3286</x:v>
+        <x:v>0.2786</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>1.3357</x:v>
+        <x:v>1.5286</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>1.5071</x:v>
+        <x:v>1.65</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.6929</x:v>
+        <x:v>1.8714</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>3.4</x:v>
+        <x:v>3.4214</x:v>
       </x:c>
       <x:c r="J25" s="0">
         <x:v>8.4429</x:v>
       </x:c>
       <x:c r="K25" s="0">
-        <x:v>2.7845</x:v>
+        <x:v>2.8655</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:11">
@@ -1386,28 +1386,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>317</x:v>
+        <x:v>315.5</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>0.8036</x:v>
+        <x:v>0.4643</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>3.7679</x:v>
+        <x:v>3.8929</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>4.1429</x:v>
+        <x:v>4.2143</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>4.6607</x:v>
+        <x:v>4.5893</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>8.9286</x:v>
+        <x:v>9.0179</x:v>
       </x:c>
       <x:c r="J26" s="0">
         <x:v>24.0179</x:v>
       </x:c>
       <x:c r="K26" s="0">
-        <x:v>7.7202</x:v>
+        <x:v>7.6994</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:11">
@@ -1421,28 +1421,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>271.25</x:v>
+        <x:v>275.5</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>0.9286</x:v>
+        <x:v>0.8214</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>3.3571</x:v>
+        <x:v>3.8571</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>3.7679</x:v>
+        <x:v>4.2143</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>4.8036</x:v>
+        <x:v>5.1071</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>11.0813</x:v>
+        <x:v>10.9821</x:v>
       </x:c>
       <x:c r="J27" s="0">
-        <x:v>22.9463</x:v>
+        <x:v>23.0713</x:v>
       </x:c>
       <x:c r="K27" s="0">
-        <x:v>7.8141</x:v>
+        <x:v>8.0089</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:11">
@@ -1456,28 +1456,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>43.44</x:v>
+        <x:v>43.6</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>0.1743</x:v>
+        <x:v>0.1071</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>0.6543</x:v>
+        <x:v>0.6886</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>0.8129</x:v>
+        <x:v>0.8514</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>1.0443</x:v>
+        <x:v>0.9914</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>2.6486</x:v>
+        <x:v>2.5286</x:v>
       </x:c>
       <x:c r="J28" s="0">
         <x:v>6.7107</x:v>
       </x:c>
       <x:c r="K28" s="0">
-        <x:v>2.0075</x:v>
+        <x:v>1.9796</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:11">
@@ -1491,28 +1491,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D29" s="0">
-        <x:v>61</x:v>
+        <x:v>61.35</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>0.2179</x:v>
+        <x:v>0.1214</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>0.7464</x:v>
+        <x:v>0.8857</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>0.8036</x:v>
+        <x:v>0.875</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>0.9071</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>2.1071</x:v>
+        <x:v>2.1464</x:v>
       </x:c>
       <x:c r="J29" s="0">
         <x:v>4.8357</x:v>
       </x:c>
       <x:c r="K29" s="0">
-        <x:v>1.603</x:v>
+        <x:v>1.644</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:11">
@@ -1526,28 +1526,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D30" s="0">
-        <x:v>251</x:v>
+        <x:v>252.5</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>1.1429</x:v>
+        <x:v>0.625</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>3.6821</x:v>
+        <x:v>3.7179</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>4.4929</x:v>
+        <x:v>4.3857</x:v>
       </x:c>
       <x:c r="H30" s="0">
-        <x:v>4.7393</x:v>
+        <x:v>4.7214</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>11.0643</x:v>
+        <x:v>10.6893</x:v>
       </x:c>
       <x:c r="J30" s="0">
         <x:v>22.2604</x:v>
       </x:c>
       <x:c r="K30" s="0">
-        <x:v>7.897</x:v>
+        <x:v>7.7333</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:11">
@@ -1561,28 +1561,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D31" s="0">
-        <x:v>33.74</x:v>
+        <x:v>33.44</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>0.1157</x:v>
+        <x:v>0.0671</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>0.4486</x:v>
+        <x:v>0.51</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>0.4857</x:v>
+        <x:v>0.5357</x:v>
       </x:c>
       <x:c r="H31" s="0">
-        <x:v>0.5514</x:v>
+        <x:v>0.5886</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>1.2857</x:v>
+        <x:v>1.3014</x:v>
       </x:c>
       <x:c r="J31" s="0">
         <x:v>3.35</x:v>
       </x:c>
       <x:c r="K31" s="0">
-        <x:v>1.0395</x:v>
+        <x:v>1.0588</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:11">
@@ -1596,28 +1596,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D32" s="0">
-        <x:v>37.54</x:v>
+        <x:v>37.38</x:v>
       </x:c>
       <x:c r="E32" s="0">
-        <x:v>0.06</x:v>
+        <x:v>0.0829</x:v>
       </x:c>
       <x:c r="F32" s="0">
-        <x:v>0.4343</x:v>
+        <x:v>0.5057</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>0.5243</x:v>
+        <x:v>0.5514</x:v>
       </x:c>
       <x:c r="H32" s="0">
-        <x:v>0.6229</x:v>
+        <x:v>0.6443</x:v>
       </x:c>
       <x:c r="I32" s="0">
-        <x:v>1.3814</x:v>
+        <x:v>1.3929</x:v>
       </x:c>
       <x:c r="J32" s="0">
-        <x:v>3.3986</x:v>
+        <x:v>3.4</x:v>
       </x:c>
       <x:c r="K32" s="0">
-        <x:v>1.0702</x:v>
+        <x:v>1.0962</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
remove: monitor_off.pyw ve ilgili tum dosyalar kaldirildi
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ATR_Sonuc.xlsx
+++ b/ATR_Sonuc.xlsx
@@ -546,28 +546,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>17.45</x:v>
+        <x:v>18.53</x:v>
       </x:c>
       <x:c r="E2" s="0">
-        <x:v>0.0321</x:v>
+        <x:v>0.0664</x:v>
       </x:c>
       <x:c r="F2" s="0">
-        <x:v>0.1864</x:v>
+        <x:v>0.1629</x:v>
       </x:c>
       <x:c r="G2" s="0">
-        <x:v>0.23</x:v>
+        <x:v>0.2736</x:v>
       </x:c>
       <x:c r="H2" s="0">
-        <x:v>0.2957</x:v>
+        <x:v>0.4243</x:v>
       </x:c>
       <x:c r="I2" s="0">
-        <x:v>0.6643</x:v>
+        <x:v>0.7393</x:v>
       </x:c>
       <x:c r="J2" s="0">
-        <x:v>1.8114</x:v>
+        <x:v>1.9464</x:v>
       </x:c>
       <x:c r="K2" s="0">
-        <x:v>0.5367</x:v>
+        <x:v>0.6021</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:11">
@@ -581,28 +581,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>75.1</x:v>
+        <x:v>77.6</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>0.175</x:v>
+        <x:v>0.2464</x:v>
       </x:c>
       <x:c r="F3" s="0">
-        <x:v>0.8607</x:v>
+        <x:v>0.6607</x:v>
       </x:c>
       <x:c r="G3" s="0">
-        <x:v>1.0786</x:v>
+        <x:v>1.2679</x:v>
       </x:c>
       <x:c r="H3" s="0">
-        <x:v>1.325</x:v>
+        <x:v>1.5143</x:v>
       </x:c>
       <x:c r="I3" s="0">
-        <x:v>2.9195</x:v>
+        <x:v>2.8357</x:v>
       </x:c>
       <x:c r="J3" s="0">
-        <x:v>7.6001</x:v>
+        <x:v>7.9504</x:v>
       </x:c>
       <x:c r="K3" s="0">
-        <x:v>2.3265</x:v>
+        <x:v>2.4126</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:11">
@@ -616,28 +616,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D4" s="0">
-        <x:v>375.25</x:v>
+        <x:v>407.25</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>1.1607</x:v>
+        <x:v>1.3036</x:v>
       </x:c>
       <x:c r="F4" s="0">
-        <x:v>6.1071</x:v>
+        <x:v>3.7143</x:v>
       </x:c>
       <x:c r="G4" s="0">
-        <x:v>6.3393</x:v>
+        <x:v>6.0536</x:v>
       </x:c>
       <x:c r="H4" s="0">
-        <x:v>6.8929</x:v>
+        <x:v>10.3929</x:v>
       </x:c>
       <x:c r="I4" s="0">
-        <x:v>13.7857</x:v>
+        <x:v>16.4286</x:v>
       </x:c>
       <x:c r="J4" s="0">
-        <x:v>32.3786</x:v>
+        <x:v>33.1786</x:v>
       </x:c>
       <x:c r="K4" s="0">
-        <x:v>11.1107</x:v>
+        <x:v>11.8452</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:11">
@@ -651,28 +651,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D5" s="0">
-        <x:v>209.1</x:v>
+        <x:v>190.5</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>0.45</x:v>
+        <x:v>0.5071</x:v>
       </x:c>
       <x:c r="F5" s="0">
-        <x:v>3.1143</x:v>
+        <x:v>2.3929</x:v>
       </x:c>
       <x:c r="G5" s="0">
-        <x:v>3.45</x:v>
+        <x:v>3.7357</x:v>
       </x:c>
       <x:c r="H5" s="0">
-        <x:v>3.8786</x:v>
+        <x:v>4.4286</x:v>
       </x:c>
       <x:c r="I5" s="0">
-        <x:v>10.3857</x:v>
+        <x:v>9.2429</x:v>
       </x:c>
       <x:c r="J5" s="0">
-        <x:v>21.4071</x:v>
+        <x:v>21.6714</x:v>
       </x:c>
       <x:c r="K5" s="0">
-        <x:v>7.1143</x:v>
+        <x:v>6.9964</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:11">
@@ -686,28 +686,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>739</x:v>
+        <x:v>744.5</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>1.5714</x:v>
+        <x:v>1.8929</x:v>
       </x:c>
       <x:c r="F6" s="0">
-        <x:v>8.3214</x:v>
+        <x:v>5.4286</x:v>
       </x:c>
       <x:c r="G6" s="0">
-        <x:v>9.4643</x:v>
+        <x:v>9.3214</x:v>
       </x:c>
       <x:c r="H6" s="0">
-        <x:v>10.7143</x:v>
+        <x:v>11.0357</x:v>
       </x:c>
       <x:c r="I6" s="0">
-        <x:v>23.8929</x:v>
+        <x:v>21.4286</x:v>
       </x:c>
       <x:c r="J6" s="0">
-        <x:v>57</x:v>
+        <x:v>55.8929</x:v>
       </x:c>
       <x:c r="K6" s="0">
-        <x:v>18.494</x:v>
+        <x:v>17.5</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -721,28 +721,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>1999</x:v>
+        <x:v>2176</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>2.7857</x:v>
+        <x:v>7.2143</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>21.7143</x:v>
+        <x:v>16.1429</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>20.2857</x:v>
+        <x:v>27.1429</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>22.3571</x:v>
+        <x:v>48.2857</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>49.7143</x:v>
+        <x:v>62.4286</x:v>
       </x:c>
       <x:c r="J7" s="0">
-        <x:v>175.4286</x:v>
+        <x:v>180.7857</x:v>
       </x:c>
       <x:c r="K7" s="0">
-        <x:v>48.7143</x:v>
+        <x:v>57</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:11">
@@ -756,28 +756,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>20.5</x:v>
+        <x:v>20.96</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>0.0443</x:v>
+        <x:v>0.0714</x:v>
       </x:c>
       <x:c r="F8" s="0">
-        <x:v>0.265</x:v>
+        <x:v>0.1871</x:v>
       </x:c>
       <x:c r="G8" s="0">
-        <x:v>0.2893</x:v>
+        <x:v>0.2743</x:v>
       </x:c>
       <x:c r="H8" s="0">
-        <x:v>0.3421</x:v>
+        <x:v>0.36</x:v>
       </x:c>
       <x:c r="I8" s="0">
-        <x:v>0.7686</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="J8" s="0">
-        <x:v>2.0614</x:v>
+        <x:v>2.0943</x:v>
       </x:c>
       <x:c r="K8" s="0">
-        <x:v>0.6285</x:v>
+        <x:v>0.6145</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
@@ -791,28 +791,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>94.75</x:v>
+        <x:v>102.9</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>0.1464</x:v>
+        <x:v>0.3571</x:v>
       </x:c>
       <x:c r="F9" s="0">
-        <x:v>1.0429</x:v>
+        <x:v>0.9643</x:v>
       </x:c>
       <x:c r="G9" s="0">
-        <x:v>1.1773</x:v>
+        <x:v>1.8929</x:v>
       </x:c>
       <x:c r="H9" s="0">
-        <x:v>1.3268</x:v>
+        <x:v>2.55</x:v>
       </x:c>
       <x:c r="I9" s="0">
-        <x:v>2.8979</x:v>
+        <x:v>3.5673</x:v>
       </x:c>
       <x:c r="J9" s="0">
-        <x:v>6.81</x:v>
+        <x:v>7.6607</x:v>
       </x:c>
       <x:c r="K9" s="0">
-        <x:v>2.2335</x:v>
+        <x:v>2.832</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:11">
@@ -826,28 +826,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>30.46</x:v>
+        <x:v>30.9</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>0.1086</x:v>
+        <x:v>0.0986</x:v>
       </x:c>
       <x:c r="F10" s="0">
-        <x:v>0.3414</x:v>
+        <x:v>0.2671</x:v>
       </x:c>
       <x:c r="G10" s="0">
-        <x:v>0.4243</x:v>
+        <x:v>0.42</x:v>
       </x:c>
       <x:c r="H10" s="0">
         <x:v>0.5943</x:v>
       </x:c>
       <x:c r="I10" s="0">
-        <x:v>1.1357</x:v>
+        <x:v>1.1514</x:v>
       </x:c>
       <x:c r="J10" s="0">
-        <x:v>2.0771</x:v>
+        <x:v>2.1886</x:v>
       </x:c>
       <x:c r="K10" s="0">
-        <x:v>0.7802</x:v>
+        <x:v>0.7867</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:11">
@@ -861,28 +861,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>102.2</x:v>
+        <x:v>105.8</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>0.2357</x:v>
+        <x:v>0.3643</x:v>
       </x:c>
       <x:c r="F11" s="0">
-        <x:v>1.1357</x:v>
+        <x:v>0.8929</x:v>
       </x:c>
       <x:c r="G11" s="0">
-        <x:v>1.1607</x:v>
+        <x:v>1.4929</x:v>
       </x:c>
       <x:c r="H11" s="0">
-        <x:v>1.3464</x:v>
+        <x:v>1.5643</x:v>
       </x:c>
       <x:c r="I11" s="0">
-        <x:v>3.4</x:v>
+        <x:v>3.0357</x:v>
       </x:c>
       <x:c r="J11" s="0">
-        <x:v>8.648</x:v>
+        <x:v>8.8419</x:v>
       </x:c>
       <x:c r="K11" s="0">
-        <x:v>2.6544</x:v>
+        <x:v>2.6986</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:11">
@@ -896,28 +896,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>136.5</x:v>
+        <x:v>136.7</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>0.2571</x:v>
+        <x:v>0.4571</x:v>
       </x:c>
       <x:c r="F12" s="0">
-        <x:v>1.8929</x:v>
+        <x:v>0.9929</x:v>
       </x:c>
       <x:c r="G12" s="0">
-        <x:v>2.1558</x:v>
+        <x:v>1.9</x:v>
       </x:c>
       <x:c r="H12" s="0">
-        <x:v>2.5225</x:v>
+        <x:v>2.1357</x:v>
       </x:c>
       <x:c r="I12" s="0">
-        <x:v>4.6531</x:v>
+        <x:v>4.5186</x:v>
       </x:c>
       <x:c r="J12" s="0">
-        <x:v>11.467</x:v>
+        <x:v>11.671</x:v>
       </x:c>
       <x:c r="K12" s="0">
-        <x:v>3.8247</x:v>
+        <x:v>3.6126</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:11">
@@ -931,28 +931,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>494.5</x:v>
+        <x:v>523</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>1.1964</x:v>
+        <x:v>1.75</x:v>
       </x:c>
       <x:c r="F13" s="0">
-        <x:v>7.5536</x:v>
+        <x:v>8.1429</x:v>
       </x:c>
       <x:c r="G13" s="0">
-        <x:v>7.9821</x:v>
+        <x:v>9.4286</x:v>
       </x:c>
       <x:c r="H13" s="0">
-        <x:v>10.5893</x:v>
+        <x:v>10.8036</x:v>
       </x:c>
       <x:c r="I13" s="0">
-        <x:v>21.6786</x:v>
+        <x:v>21.0357</x:v>
       </x:c>
       <x:c r="J13" s="0">
-        <x:v>52.75</x:v>
+        <x:v>55.5714</x:v>
       </x:c>
       <x:c r="K13" s="0">
-        <x:v>16.9583</x:v>
+        <x:v>17.7887</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:11">
@@ -966,28 +966,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>14.15</x:v>
+        <x:v>14.34</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>0.0357</x:v>
+        <x:v>0.05</x:v>
       </x:c>
       <x:c r="F14" s="0">
-        <x:v>0.2121</x:v>
+        <x:v>0.1179</x:v>
       </x:c>
       <x:c r="G14" s="0">
-        <x:v>0.2214</x:v>
+        <x:v>0.2114</x:v>
       </x:c>
       <x:c r="H14" s="0">
-        <x:v>0.2371</x:v>
+        <x:v>0.2307</x:v>
       </x:c>
       <x:c r="I14" s="0">
-        <x:v>0.4917</x:v>
+        <x:v>0.4895</x:v>
       </x:c>
       <x:c r="J14" s="0">
-        <x:v>1.2753</x:v>
+        <x:v>1.3345</x:v>
       </x:c>
       <x:c r="K14" s="0">
-        <x:v>0.4122</x:v>
+        <x:v>0.4057</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:11">
@@ -1001,28 +1001,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>200.3</x:v>
+        <x:v>203.1</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>0.3214</x:v>
+        <x:v>0.7</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>2.3786</x:v>
+        <x:v>1.5357</x:v>
       </x:c>
       <x:c r="G15" s="0">
-        <x:v>2.6571</x:v>
+        <x:v>2.2429</x:v>
       </x:c>
       <x:c r="H15" s="0">
-        <x:v>2.7643</x:v>
+        <x:v>2.8143</x:v>
       </x:c>
       <x:c r="I15" s="0">
-        <x:v>6.0816</x:v>
+        <x:v>5.9571</x:v>
       </x:c>
       <x:c r="J15" s="0">
-        <x:v>13.9501</x:v>
+        <x:v>14.0085</x:v>
       </x:c>
       <x:c r="K15" s="0">
-        <x:v>4.6922</x:v>
+        <x:v>4.5431</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:11">
@@ -1036,28 +1036,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>36.84</x:v>
+        <x:v>35.74</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>0.1729</x:v>
+        <x:v>0.1429</x:v>
       </x:c>
       <x:c r="F16" s="0">
-        <x:v>0.7114</x:v>
+        <x:v>0.4743</x:v>
       </x:c>
       <x:c r="G16" s="0">
-        <x:v>0.7329</x:v>
+        <x:v>0.6286</x:v>
       </x:c>
       <x:c r="H16" s="0">
-        <x:v>0.93</x:v>
+        <x:v>0.9014</x:v>
       </x:c>
       <x:c r="I16" s="0">
-        <x:v>1.5771</x:v>
+        <x:v>1.7743</x:v>
       </x:c>
       <x:c r="J16" s="0">
-        <x:v>2.7871</x:v>
+        <x:v>2.9114</x:v>
       </x:c>
       <x:c r="K16" s="0">
-        <x:v>1.1519</x:v>
+        <x:v>1.1388</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:11">
@@ -1071,28 +1071,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D17" s="0">
-        <x:v>646</x:v>
+        <x:v>658</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>1.3214</x:v>
+        <x:v>1.4286</x:v>
       </x:c>
       <x:c r="F17" s="0">
-        <x:v>7.8571</x:v>
+        <x:v>3.8929</x:v>
       </x:c>
       <x:c r="G17" s="0">
-        <x:v>8.3214</x:v>
+        <x:v>7.1071</x:v>
       </x:c>
       <x:c r="H17" s="0">
-        <x:v>9.4286</x:v>
+        <x:v>10.0357</x:v>
       </x:c>
       <x:c r="I17" s="0">
-        <x:v>19.9643</x:v>
+        <x:v>17.8929</x:v>
       </x:c>
       <x:c r="J17" s="0">
-        <x:v>51.1429</x:v>
+        <x:v>49</x:v>
       </x:c>
       <x:c r="K17" s="0">
-        <x:v>16.3393</x:v>
+        <x:v>14.8929</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:11">
@@ -1106,28 +1106,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>42.14</x:v>
+        <x:v>39.44</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>0.0829</x:v>
+        <x:v>0.1014</x:v>
       </x:c>
       <x:c r="F18" s="0">
-        <x:v>0.6071</x:v>
+        <x:v>0.3257</x:v>
       </x:c>
       <x:c r="G18" s="0">
-        <x:v>0.7514</x:v>
+        <x:v>0.4771</x:v>
       </x:c>
       <x:c r="H18" s="0">
-        <x:v>0.9129</x:v>
+        <x:v>0.7671</x:v>
       </x:c>
       <x:c r="I18" s="0">
-        <x:v>2.1971</x:v>
+        <x:v>2.1914</x:v>
       </x:c>
       <x:c r="J18" s="0">
-        <x:v>4.3829</x:v>
+        <x:v>4.4529</x:v>
       </x:c>
       <x:c r="K18" s="0">
-        <x:v>1.489</x:v>
+        <x:v>1.386</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:11">
@@ -1141,28 +1141,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D19" s="0">
-        <x:v>20.94</x:v>
+        <x:v>22.64</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>0.0629</x:v>
+        <x:v>0.0743</x:v>
       </x:c>
       <x:c r="F19" s="0">
-        <x:v>0.3557</x:v>
+        <x:v>0.2557</x:v>
       </x:c>
       <x:c r="G19" s="0">
-        <x:v>0.4529</x:v>
+        <x:v>0.3386</x:v>
       </x:c>
       <x:c r="H19" s="0">
-        <x:v>0.5179</x:v>
+        <x:v>0.4671</x:v>
       </x:c>
       <x:c r="I19" s="0">
-        <x:v>1.2571</x:v>
+        <x:v>1.1093</x:v>
       </x:c>
       <x:c r="J19" s="0">
-        <x:v>1.8579</x:v>
+        <x:v>1.9257</x:v>
       </x:c>
       <x:c r="K19" s="0">
-        <x:v>0.7507</x:v>
+        <x:v>0.6951</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:11">
@@ -1176,28 +1176,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D20" s="0">
-        <x:v>184.5</x:v>
+        <x:v>185.4</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>0.2643</x:v>
+        <x:v>0.45</x:v>
       </x:c>
       <x:c r="F20" s="0">
-        <x:v>2.3143</x:v>
+        <x:v>1.3929</x:v>
       </x:c>
       <x:c r="G20" s="0">
-        <x:v>2.45</x:v>
+        <x:v>2.1143</x:v>
       </x:c>
       <x:c r="H20" s="0">
-        <x:v>2.6786</x:v>
+        <x:v>2.4286</x:v>
       </x:c>
       <x:c r="I20" s="0">
-        <x:v>5.25</x:v>
+        <x:v>5.0571</x:v>
       </x:c>
       <x:c r="J20" s="0">
-        <x:v>13.6286</x:v>
+        <x:v>13.1071</x:v>
       </x:c>
       <x:c r="K20" s="0">
-        <x:v>4.431</x:v>
+        <x:v>4.0917</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:11">
@@ -1211,28 +1211,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>97.3</x:v>
+        <x:v>99.15</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>0.2429</x:v>
+        <x:v>0.3107</x:v>
       </x:c>
       <x:c r="F21" s="0">
-        <x:v>1.4036</x:v>
+        <x:v>0.8321</x:v>
       </x:c>
       <x:c r="G21" s="0">
-        <x:v>1.5464</x:v>
+        <x:v>1.2571</x:v>
       </x:c>
       <x:c r="H21" s="0">
-        <x:v>1.7786</x:v>
+        <x:v>1.6464</x:v>
       </x:c>
       <x:c r="I21" s="0">
-        <x:v>3.4332</x:v>
+        <x:v>3.4249</x:v>
       </x:c>
       <x:c r="J21" s="0">
-        <x:v>8.2544</x:v>
+        <x:v>8.5027</x:v>
       </x:c>
       <x:c r="K21" s="0">
-        <x:v>2.7765</x:v>
+        <x:v>2.6623</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:11">
@@ -1246,28 +1246,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>2.46</x:v>
+        <x:v>3.03</x:v>
       </x:c>
       <x:c r="E22" s="0">
-        <x:v>0.0136</x:v>
+        <x:v>0.0236</x:v>
       </x:c>
       <x:c r="F22" s="0">
-        <x:v>0.0329</x:v>
+        <x:v>0.065</x:v>
       </x:c>
       <x:c r="G22" s="0">
-        <x:v>0.0357</x:v>
+        <x:v>0.0814</x:v>
       </x:c>
       <x:c r="H22" s="0">
-        <x:v>0.0514</x:v>
+        <x:v>0.0936</x:v>
       </x:c>
       <x:c r="I22" s="0">
-        <x:v>0.1</x:v>
+        <x:v>0.1314</x:v>
       </x:c>
       <x:c r="J22" s="0">
-        <x:v>0.2714</x:v>
+        <x:v>0.2764</x:v>
       </x:c>
       <x:c r="K22" s="0">
-        <x:v>0.0842</x:v>
+        <x:v>0.1119</x:v>
       </x:c>
     </x:row>
     <x:row r="23" spans="1:11">
@@ -1281,28 +1281,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>46.4</x:v>
+        <x:v>46.88</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>0.1086</x:v>
+        <x:v>0.1229</x:v>
       </x:c>
       <x:c r="F23" s="0">
-        <x:v>0.6814</x:v>
+        <x:v>0.4329</x:v>
       </x:c>
       <x:c r="G23" s="0">
-        <x:v>0.76</x:v>
+        <x:v>0.6043</x:v>
       </x:c>
       <x:c r="H23" s="0">
-        <x:v>0.7986</x:v>
+        <x:v>0.6957</x:v>
       </x:c>
       <x:c r="I23" s="0">
-        <x:v>2.1186</x:v>
+        <x:v>1.64</x:v>
       </x:c>
       <x:c r="J23" s="0">
-        <x:v>4.2871</x:v>
+        <x:v>4.3586</x:v>
       </x:c>
       <x:c r="K23" s="0">
-        <x:v>1.459</x:v>
+        <x:v>1.309</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:11">
@@ -1316,28 +1316,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>337.75</x:v>
+        <x:v>314.25</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>0.6429</x:v>
+        <x:v>1.0357</x:v>
       </x:c>
       <x:c r="F24" s="0">
-        <x:v>5.3393</x:v>
+        <x:v>3.4821</x:v>
       </x:c>
       <x:c r="G24" s="0">
-        <x:v>5.9643</x:v>
+        <x:v>5.1429</x:v>
       </x:c>
       <x:c r="H24" s="0">
-        <x:v>7.1071</x:v>
+        <x:v>6.7321</x:v>
       </x:c>
       <x:c r="I24" s="0">
-        <x:v>14.7143</x:v>
+        <x:v>14.2857</x:v>
       </x:c>
       <x:c r="J24" s="0">
-        <x:v>27.7143</x:v>
+        <x:v>29.2679</x:v>
       </x:c>
       <x:c r="K24" s="0">
-        <x:v>10.247</x:v>
+        <x:v>9.9911</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:11">
@@ -1351,28 +1351,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>112.3</x:v>
+        <x:v>116.9</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>0.2786</x:v>
+        <x:v>0.2714</x:v>
       </x:c>
       <x:c r="F25" s="0">
-        <x:v>1.5286</x:v>
+        <x:v>0.7571</x:v>
       </x:c>
       <x:c r="G25" s="0">
-        <x:v>1.65</x:v>
+        <x:v>1.25</x:v>
       </x:c>
       <x:c r="H25" s="0">
-        <x:v>1.8714</x:v>
+        <x:v>1.6286</x:v>
       </x:c>
       <x:c r="I25" s="0">
-        <x:v>3.4214</x:v>
+        <x:v>3.3143</x:v>
       </x:c>
       <x:c r="J25" s="0">
-        <x:v>8.4429</x:v>
+        <x:v>8.8607</x:v>
       </x:c>
       <x:c r="K25" s="0">
-        <x:v>2.8655</x:v>
+        <x:v>2.6804</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:11">
@@ -1386,28 +1386,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D26" s="0">
-        <x:v>315.5</x:v>
+        <x:v>316.5</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>0.4643</x:v>
+        <x:v>0.7143</x:v>
       </x:c>
       <x:c r="F26" s="0">
-        <x:v>3.8929</x:v>
+        <x:v>2.1786</x:v>
       </x:c>
       <x:c r="G26" s="0">
-        <x:v>4.2143</x:v>
+        <x:v>3.5893</x:v>
       </x:c>
       <x:c r="H26" s="0">
-        <x:v>4.5893</x:v>
+        <x:v>4.2321</x:v>
       </x:c>
       <x:c r="I26" s="0">
-        <x:v>9.0179</x:v>
+        <x:v>9.375</x:v>
       </x:c>
       <x:c r="J26" s="0">
-        <x:v>24.0179</x:v>
+        <x:v>23.3929</x:v>
       </x:c>
       <x:c r="K26" s="0">
-        <x:v>7.6994</x:v>
+        <x:v>7.247</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:11">
@@ -1421,28 +1421,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>275.5</x:v>
+        <x:v>286.5</x:v>
       </x:c>
       <x:c r="E27" s="0">
-        <x:v>0.8214</x:v>
+        <x:v>1.0714</x:v>
       </x:c>
       <x:c r="F27" s="0">
-        <x:v>3.8571</x:v>
+        <x:v>3.3036</x:v>
       </x:c>
       <x:c r="G27" s="0">
-        <x:v>4.2143</x:v>
+        <x:v>5.1786</x:v>
       </x:c>
       <x:c r="H27" s="0">
-        <x:v>5.1071</x:v>
+        <x:v>5.6786</x:v>
       </x:c>
       <x:c r="I27" s="0">
-        <x:v>10.9821</x:v>
+        <x:v>10.8036</x:v>
       </x:c>
       <x:c r="J27" s="0">
-        <x:v>23.0713</x:v>
+        <x:v>23.8805</x:v>
       </x:c>
       <x:c r="K27" s="0">
-        <x:v>8.0089</x:v>
+        <x:v>8.3194</x:v>
       </x:c>
     </x:row>
     <x:row r="28" spans="1:11">
@@ -1456,28 +1456,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>43.6</x:v>
+        <x:v>46.2</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>0.1071</x:v>
+        <x:v>0.1914</x:v>
       </x:c>
       <x:c r="F28" s="0">
-        <x:v>0.6886</x:v>
+        <x:v>0.68</x:v>
       </x:c>
       <x:c r="G28" s="0">
-        <x:v>0.8514</x:v>
+        <x:v>1.0157</x:v>
       </x:c>
       <x:c r="H28" s="0">
-        <x:v>0.9914</x:v>
+        <x:v>1.03</x:v>
       </x:c>
       <x:c r="I28" s="0">
-        <x:v>2.5286</x:v>
+        <x:v>2.3029</x:v>
       </x:c>
       <x:c r="J28" s="0">
-        <x:v>6.7107</x:v>
+        <x:v>6.7721</x:v>
       </x:c>
       <x:c r="K28" s="0">
-        <x:v>1.9796</x:v>
+        <x:v>1.9987</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:11">
@@ -1491,28 +1491,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D29" s="0">
-        <x:v>61.35</x:v>
+        <x:v>62.75</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>0.1214</x:v>
+        <x:v>0.2143</x:v>
       </x:c>
       <x:c r="F29" s="0">
-        <x:v>0.8857</x:v>
+        <x:v>0.5536</x:v>
       </x:c>
       <x:c r="G29" s="0">
-        <x:v>0.875</x:v>
+        <x:v>0.7679</x:v>
       </x:c>
       <x:c r="H29" s="0">
-        <x:v>1</x:v>
+        <x:v>0.9964</x:v>
       </x:c>
       <x:c r="I29" s="0">
-        <x:v>2.1464</x:v>
+        <x:v>1.9607</x:v>
       </x:c>
       <x:c r="J29" s="0">
-        <x:v>4.8357</x:v>
+        <x:v>5.0071</x:v>
       </x:c>
       <x:c r="K29" s="0">
-        <x:v>1.644</x:v>
+        <x:v>1.5833</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:11">
@@ -1526,28 +1526,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D30" s="0">
-        <x:v>252.5</x:v>
+        <x:v>266.25</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>0.625</x:v>
+        <x:v>0.6964</x:v>
       </x:c>
       <x:c r="F30" s="0">
-        <x:v>3.7179</x:v>
+        <x:v>1.8393</x:v>
       </x:c>
       <x:c r="G30" s="0">
-        <x:v>4.3857</x:v>
+        <x:v>3.4286</x:v>
       </x:c>
       <x:c r="H30" s="0">
-        <x:v>4.7214</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="I30" s="0">
-        <x:v>10.6893</x:v>
+        <x:v>9.7357</x:v>
       </x:c>
       <x:c r="J30" s="0">
-        <x:v>22.2604</x:v>
+        <x:v>22.5032</x:v>
       </x:c>
       <x:c r="K30" s="0">
-        <x:v>7.7333</x:v>
+        <x:v>7.0339</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:11">
@@ -1561,28 +1561,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D31" s="0">
-        <x:v>33.44</x:v>
+        <x:v>33.6</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>0.0671</x:v>
+        <x:v>0.0914</x:v>
       </x:c>
       <x:c r="F31" s="0">
-        <x:v>0.51</x:v>
+        <x:v>0.26</x:v>
       </x:c>
       <x:c r="G31" s="0">
-        <x:v>0.5357</x:v>
+        <x:v>0.42</x:v>
       </x:c>
       <x:c r="H31" s="0">
-        <x:v>0.5886</x:v>
+        <x:v>0.5414</x:v>
       </x:c>
       <x:c r="I31" s="0">
-        <x:v>1.3014</x:v>
+        <x:v>1.1729</x:v>
       </x:c>
       <x:c r="J31" s="0">
-        <x:v>3.35</x:v>
+        <x:v>3.3557</x:v>
       </x:c>
       <x:c r="K31" s="0">
-        <x:v>1.0588</x:v>
+        <x:v>0.9736</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:11">
@@ -1596,28 +1596,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D32" s="0">
-        <x:v>37.38</x:v>
+        <x:v>37.32</x:v>
       </x:c>
       <x:c r="E32" s="0">
-        <x:v>0.0829</x:v>
+        <x:v>0.0914</x:v>
       </x:c>
       <x:c r="F32" s="0">
-        <x:v>0.5057</x:v>
+        <x:v>0.2471</x:v>
       </x:c>
       <x:c r="G32" s="0">
-        <x:v>0.5514</x:v>
+        <x:v>0.5229</x:v>
       </x:c>
       <x:c r="H32" s="0">
-        <x:v>0.6443</x:v>
+        <x:v>0.6114</x:v>
       </x:c>
       <x:c r="I32" s="0">
-        <x:v>1.3929</x:v>
+        <x:v>1.3071</x:v>
       </x:c>
       <x:c r="J32" s="0">
-        <x:v>3.4</x:v>
+        <x:v>3.5214</x:v>
       </x:c>
       <x:c r="K32" s="0">
-        <x:v>1.0962</x:v>
+        <x:v>1.0502</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
remove: monitor_off.pyw kalici olarak kaldirildi
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/ATR_Sonuc.xlsx
+++ b/ATR_Sonuc.xlsx
@@ -546,7 +546,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D2" s="0">
-        <x:v>18.53</x:v>
+        <x:v>18.54</x:v>
       </x:c>
       <x:c r="E2" s="0">
         <x:v>0.0664</x:v>
@@ -581,10 +581,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D3" s="0">
-        <x:v>77.6</x:v>
+        <x:v>77.7</x:v>
       </x:c>
       <x:c r="E3" s="0">
-        <x:v>0.2464</x:v>
+        <x:v>0.2536</x:v>
       </x:c>
       <x:c r="F3" s="0">
         <x:v>0.6607</x:v>
@@ -602,7 +602,7 @@
         <x:v>7.9504</x:v>
       </x:c>
       <x:c r="K3" s="0">
-        <x:v>2.4126</x:v>
+        <x:v>2.4138</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:11">
@@ -619,7 +619,7 @@
         <x:v>407.25</x:v>
       </x:c>
       <x:c r="E4" s="0">
-        <x:v>1.3036</x:v>
+        <x:v>1.3571</x:v>
       </x:c>
       <x:c r="F4" s="0">
         <x:v>3.7143</x:v>
@@ -637,7 +637,7 @@
         <x:v>33.1786</x:v>
       </x:c>
       <x:c r="K4" s="0">
-        <x:v>11.8452</x:v>
+        <x:v>11.8542</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:11">
@@ -654,7 +654,7 @@
         <x:v>190.5</x:v>
       </x:c>
       <x:c r="E5" s="0">
-        <x:v>0.5071</x:v>
+        <x:v>0.5357</x:v>
       </x:c>
       <x:c r="F5" s="0">
         <x:v>2.3929</x:v>
@@ -672,7 +672,7 @@
         <x:v>21.6714</x:v>
       </x:c>
       <x:c r="K5" s="0">
-        <x:v>6.9964</x:v>
+        <x:v>7.0012</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:11">
@@ -686,10 +686,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D6" s="0">
-        <x:v>744.5</x:v>
+        <x:v>746.5</x:v>
       </x:c>
       <x:c r="E6" s="0">
-        <x:v>1.8929</x:v>
+        <x:v>1.9643</x:v>
       </x:c>
       <x:c r="F6" s="0">
         <x:v>5.4286</x:v>
@@ -707,7 +707,7 @@
         <x:v>55.8929</x:v>
       </x:c>
       <x:c r="K6" s="0">
-        <x:v>17.5</x:v>
+        <x:v>17.5119</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:11">
@@ -721,28 +721,28 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D7" s="0">
-        <x:v>2176</x:v>
+        <x:v>2182</x:v>
       </x:c>
       <x:c r="E7" s="0">
-        <x:v>7.2143</x:v>
+        <x:v>7.7143</x:v>
       </x:c>
       <x:c r="F7" s="0">
-        <x:v>16.1429</x:v>
+        <x:v>16.6429</x:v>
       </x:c>
       <x:c r="G7" s="0">
-        <x:v>27.1429</x:v>
+        <x:v>27.6429</x:v>
       </x:c>
       <x:c r="H7" s="0">
-        <x:v>48.2857</x:v>
+        <x:v>48.7857</x:v>
       </x:c>
       <x:c r="I7" s="0">
-        <x:v>62.4286</x:v>
+        <x:v>62.9286</x:v>
       </x:c>
       <x:c r="J7" s="0">
         <x:v>180.7857</x:v>
       </x:c>
       <x:c r="K7" s="0">
-        <x:v>57</x:v>
+        <x:v>57.4167</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:11">
@@ -756,10 +756,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D8" s="0">
-        <x:v>20.96</x:v>
+        <x:v>21</x:v>
       </x:c>
       <x:c r="E8" s="0">
-        <x:v>0.0714</x:v>
+        <x:v>0.0729</x:v>
       </x:c>
       <x:c r="F8" s="0">
         <x:v>0.1871</x:v>
@@ -777,7 +777,7 @@
         <x:v>2.0943</x:v>
       </x:c>
       <x:c r="K8" s="0">
-        <x:v>0.6145</x:v>
+        <x:v>0.6148</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:11">
@@ -791,10 +791,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D9" s="0">
-        <x:v>102.9</x:v>
+        <x:v>103</x:v>
       </x:c>
       <x:c r="E9" s="0">
-        <x:v>0.3571</x:v>
+        <x:v>0.3643</x:v>
       </x:c>
       <x:c r="F9" s="0">
         <x:v>0.9643</x:v>
@@ -812,7 +812,7 @@
         <x:v>7.6607</x:v>
       </x:c>
       <x:c r="K9" s="0">
-        <x:v>2.832</x:v>
+        <x:v>2.8332</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:11">
@@ -826,10 +826,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D10" s="0">
-        <x:v>30.9</x:v>
+        <x:v>30.94</x:v>
       </x:c>
       <x:c r="E10" s="0">
-        <x:v>0.0986</x:v>
+        <x:v>0.1</x:v>
       </x:c>
       <x:c r="F10" s="0">
         <x:v>0.2671</x:v>
@@ -847,7 +847,7 @@
         <x:v>2.1886</x:v>
       </x:c>
       <x:c r="K10" s="0">
-        <x:v>0.7867</x:v>
+        <x:v>0.7869</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:11">
@@ -861,10 +861,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D11" s="0">
-        <x:v>105.8</x:v>
+        <x:v>105.9</x:v>
       </x:c>
       <x:c r="E11" s="0">
-        <x:v>0.3643</x:v>
+        <x:v>0.3714</x:v>
       </x:c>
       <x:c r="F11" s="0">
         <x:v>0.8929</x:v>
@@ -882,7 +882,7 @@
         <x:v>8.8419</x:v>
       </x:c>
       <x:c r="K11" s="0">
-        <x:v>2.6986</x:v>
+        <x:v>2.6998</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:11">
@@ -896,10 +896,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D12" s="0">
-        <x:v>136.7</x:v>
+        <x:v>136.9</x:v>
       </x:c>
       <x:c r="E12" s="0">
-        <x:v>0.4571</x:v>
+        <x:v>0.4643</x:v>
       </x:c>
       <x:c r="F12" s="0">
         <x:v>0.9929</x:v>
@@ -917,7 +917,7 @@
         <x:v>11.671</x:v>
       </x:c>
       <x:c r="K12" s="0">
-        <x:v>3.6126</x:v>
+        <x:v>3.6137</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:11">
@@ -931,10 +931,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D13" s="0">
-        <x:v>523</x:v>
+        <x:v>522</x:v>
       </x:c>
       <x:c r="E13" s="0">
-        <x:v>1.75</x:v>
+        <x:v>1.7857</x:v>
       </x:c>
       <x:c r="F13" s="0">
         <x:v>8.1429</x:v>
@@ -952,7 +952,7 @@
         <x:v>55.5714</x:v>
       </x:c>
       <x:c r="K13" s="0">
-        <x:v>17.7887</x:v>
+        <x:v>17.7946</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:11">
@@ -966,10 +966,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D14" s="0">
-        <x:v>14.34</x:v>
+        <x:v>14.37</x:v>
       </x:c>
       <x:c r="E14" s="0">
-        <x:v>0.05</x:v>
+        <x:v>0.0514</x:v>
       </x:c>
       <x:c r="F14" s="0">
         <x:v>0.1179</x:v>
@@ -987,7 +987,7 @@
         <x:v>1.3345</x:v>
       </x:c>
       <x:c r="K14" s="0">
-        <x:v>0.4057</x:v>
+        <x:v>0.4059</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:11">
@@ -1001,13 +1001,13 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D15" s="0">
-        <x:v>203.1</x:v>
+        <x:v>203.3</x:v>
       </x:c>
       <x:c r="E15" s="0">
-        <x:v>0.7</x:v>
+        <x:v>0.7214</x:v>
       </x:c>
       <x:c r="F15" s="0">
-        <x:v>1.5357</x:v>
+        <x:v>1.5429</x:v>
       </x:c>
       <x:c r="G15" s="0">
         <x:v>2.2429</x:v>
@@ -1022,7 +1022,7 @@
         <x:v>14.0085</x:v>
       </x:c>
       <x:c r="K15" s="0">
-        <x:v>4.5431</x:v>
+        <x:v>4.5478</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:11">
@@ -1036,10 +1036,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D16" s="0">
-        <x:v>35.74</x:v>
+        <x:v>35.78</x:v>
       </x:c>
       <x:c r="E16" s="0">
-        <x:v>0.1429</x:v>
+        <x:v>0.1486</x:v>
       </x:c>
       <x:c r="F16" s="0">
         <x:v>0.4743</x:v>
@@ -1057,7 +1057,7 @@
         <x:v>2.9114</x:v>
       </x:c>
       <x:c r="K16" s="0">
-        <x:v>1.1388</x:v>
+        <x:v>1.1398</x:v>
       </x:c>
     </x:row>
     <x:row r="17" spans="1:11">
@@ -1074,7 +1074,7 @@
         <x:v>658</x:v>
       </x:c>
       <x:c r="E17" s="0">
-        <x:v>1.4286</x:v>
+        <x:v>1.4643</x:v>
       </x:c>
       <x:c r="F17" s="0">
         <x:v>3.8929</x:v>
@@ -1092,7 +1092,7 @@
         <x:v>49</x:v>
       </x:c>
       <x:c r="K17" s="0">
-        <x:v>14.8929</x:v>
+        <x:v>14.8988</x:v>
       </x:c>
     </x:row>
     <x:row r="18" spans="1:11">
@@ -1106,10 +1106,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D18" s="0">
-        <x:v>39.44</x:v>
+        <x:v>39.46</x:v>
       </x:c>
       <x:c r="E18" s="0">
-        <x:v>0.1014</x:v>
+        <x:v>0.1043</x:v>
       </x:c>
       <x:c r="F18" s="0">
         <x:v>0.3257</x:v>
@@ -1127,7 +1127,7 @@
         <x:v>4.4529</x:v>
       </x:c>
       <x:c r="K18" s="0">
-        <x:v>1.386</x:v>
+        <x:v>1.3864</x:v>
       </x:c>
     </x:row>
     <x:row r="19" spans="1:11">
@@ -1144,7 +1144,7 @@
         <x:v>22.64</x:v>
       </x:c>
       <x:c r="E19" s="0">
-        <x:v>0.0743</x:v>
+        <x:v>0.0771</x:v>
       </x:c>
       <x:c r="F19" s="0">
         <x:v>0.2557</x:v>
@@ -1162,7 +1162,7 @@
         <x:v>1.9257</x:v>
       </x:c>
       <x:c r="K19" s="0">
-        <x:v>0.6951</x:v>
+        <x:v>0.6956</x:v>
       </x:c>
     </x:row>
     <x:row r="20" spans="1:11">
@@ -1179,7 +1179,7 @@
         <x:v>185.4</x:v>
       </x:c>
       <x:c r="E20" s="0">
-        <x:v>0.45</x:v>
+        <x:v>0.4571</x:v>
       </x:c>
       <x:c r="F20" s="0">
         <x:v>1.3929</x:v>
@@ -1197,7 +1197,7 @@
         <x:v>13.1071</x:v>
       </x:c>
       <x:c r="K20" s="0">
-        <x:v>4.0917</x:v>
+        <x:v>4.0929</x:v>
       </x:c>
     </x:row>
     <x:row r="21" spans="1:11">
@@ -1211,10 +1211,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D21" s="0">
-        <x:v>99.15</x:v>
+        <x:v>99.2</x:v>
       </x:c>
       <x:c r="E21" s="0">
-        <x:v>0.3107</x:v>
+        <x:v>0.3179</x:v>
       </x:c>
       <x:c r="F21" s="0">
         <x:v>0.8321</x:v>
@@ -1232,7 +1232,7 @@
         <x:v>8.5027</x:v>
       </x:c>
       <x:c r="K21" s="0">
-        <x:v>2.6623</x:v>
+        <x:v>2.6635</x:v>
       </x:c>
     </x:row>
     <x:row r="22" spans="1:11">
@@ -1246,7 +1246,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D22" s="0">
-        <x:v>3.03</x:v>
+        <x:v>3.02</x:v>
       </x:c>
       <x:c r="E22" s="0">
         <x:v>0.0236</x:v>
@@ -1281,10 +1281,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D23" s="0">
-        <x:v>46.88</x:v>
+        <x:v>46.86</x:v>
       </x:c>
       <x:c r="E23" s="0">
-        <x:v>0.1229</x:v>
+        <x:v>0.1271</x:v>
       </x:c>
       <x:c r="F23" s="0">
         <x:v>0.4329</x:v>
@@ -1302,7 +1302,7 @@
         <x:v>4.3586</x:v>
       </x:c>
       <x:c r="K23" s="0">
-        <x:v>1.309</x:v>
+        <x:v>1.3098</x:v>
       </x:c>
     </x:row>
     <x:row r="24" spans="1:11">
@@ -1316,10 +1316,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D24" s="0">
-        <x:v>314.25</x:v>
+        <x:v>314.5</x:v>
       </x:c>
       <x:c r="E24" s="0">
-        <x:v>1.0357</x:v>
+        <x:v>1.0536</x:v>
       </x:c>
       <x:c r="F24" s="0">
         <x:v>3.4821</x:v>
@@ -1337,7 +1337,7 @@
         <x:v>29.2679</x:v>
       </x:c>
       <x:c r="K24" s="0">
-        <x:v>9.9911</x:v>
+        <x:v>9.994</x:v>
       </x:c>
     </x:row>
     <x:row r="25" spans="1:11">
@@ -1351,10 +1351,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D25" s="0">
-        <x:v>116.9</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="E25" s="0">
-        <x:v>0.2714</x:v>
+        <x:v>0.2786</x:v>
       </x:c>
       <x:c r="F25" s="0">
         <x:v>0.7571</x:v>
@@ -1372,7 +1372,7 @@
         <x:v>8.8607</x:v>
       </x:c>
       <x:c r="K25" s="0">
-        <x:v>2.6804</x:v>
+        <x:v>2.6815</x:v>
       </x:c>
     </x:row>
     <x:row r="26" spans="1:11">
@@ -1389,7 +1389,7 @@
         <x:v>316.5</x:v>
       </x:c>
       <x:c r="E26" s="0">
-        <x:v>0.7143</x:v>
+        <x:v>0.7321</x:v>
       </x:c>
       <x:c r="F26" s="0">
         <x:v>2.1786</x:v>
@@ -1407,7 +1407,7 @@
         <x:v>23.3929</x:v>
       </x:c>
       <x:c r="K26" s="0">
-        <x:v>7.247</x:v>
+        <x:v>7.25</x:v>
       </x:c>
     </x:row>
     <x:row r="27" spans="1:11">
@@ -1421,7 +1421,7 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D27" s="0">
-        <x:v>286.5</x:v>
+        <x:v>286.75</x:v>
       </x:c>
       <x:c r="E27" s="0">
         <x:v>1.0714</x:v>
@@ -1456,10 +1456,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D28" s="0">
-        <x:v>46.2</x:v>
+        <x:v>46.24</x:v>
       </x:c>
       <x:c r="E28" s="0">
-        <x:v>0.1914</x:v>
+        <x:v>0.1929</x:v>
       </x:c>
       <x:c r="F28" s="0">
         <x:v>0.68</x:v>
@@ -1477,7 +1477,7 @@
         <x:v>6.7721</x:v>
       </x:c>
       <x:c r="K28" s="0">
-        <x:v>1.9987</x:v>
+        <x:v>1.9989</x:v>
       </x:c>
     </x:row>
     <x:row r="29" spans="1:11">
@@ -1491,10 +1491,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D29" s="0">
-        <x:v>62.75</x:v>
+        <x:v>62.8</x:v>
       </x:c>
       <x:c r="E29" s="0">
-        <x:v>0.2143</x:v>
+        <x:v>0.2179</x:v>
       </x:c>
       <x:c r="F29" s="0">
         <x:v>0.5536</x:v>
@@ -1512,7 +1512,7 @@
         <x:v>5.0071</x:v>
       </x:c>
       <x:c r="K29" s="0">
-        <x:v>1.5833</x:v>
+        <x:v>1.5839</x:v>
       </x:c>
     </x:row>
     <x:row r="30" spans="1:11">
@@ -1526,10 +1526,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D30" s="0">
-        <x:v>266.25</x:v>
+        <x:v>266.75</x:v>
       </x:c>
       <x:c r="E30" s="0">
-        <x:v>0.6964</x:v>
+        <x:v>0.7143</x:v>
       </x:c>
       <x:c r="F30" s="0">
         <x:v>1.8393</x:v>
@@ -1547,7 +1547,7 @@
         <x:v>22.5032</x:v>
       </x:c>
       <x:c r="K30" s="0">
-        <x:v>7.0339</x:v>
+        <x:v>7.0368</x:v>
       </x:c>
     </x:row>
     <x:row r="31" spans="1:11">
@@ -1561,10 +1561,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D31" s="0">
-        <x:v>33.6</x:v>
+        <x:v>33.66</x:v>
       </x:c>
       <x:c r="E31" s="0">
-        <x:v>0.0914</x:v>
+        <x:v>0.0929</x:v>
       </x:c>
       <x:c r="F31" s="0">
         <x:v>0.26</x:v>
@@ -1582,7 +1582,7 @@
         <x:v>3.3557</x:v>
       </x:c>
       <x:c r="K31" s="0">
-        <x:v>0.9736</x:v>
+        <x:v>0.9738</x:v>
       </x:c>
     </x:row>
     <x:row r="32" spans="1:11">
@@ -1596,10 +1596,10 @@
         <x:v>13</x:v>
       </x:c>
       <x:c r="D32" s="0">
-        <x:v>37.32</x:v>
+        <x:v>37.34</x:v>
       </x:c>
       <x:c r="E32" s="0">
-        <x:v>0.0914</x:v>
+        <x:v>0.0929</x:v>
       </x:c>
       <x:c r="F32" s="0">
         <x:v>0.2471</x:v>
@@ -1617,7 +1617,7 @@
         <x:v>3.5214</x:v>
       </x:c>
       <x:c r="K32" s="0">
-        <x:v>1.0502</x:v>
+        <x:v>1.0505</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>